<commit_message>
se actualiza archivos 21_04_2026
</commit_message>
<xml_diff>
--- a/DataSphere/Encuestas Satisfaccion/Formato Objetos Transporte Ajustes Encuestas Satisfacción.xlsx
+++ b/DataSphere/Encuestas Satisfaccion/Formato Objetos Transporte Ajustes Encuestas Satisfacción.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\degonzalez\Documents\2026\Backup_2026\DataSphere\Encuestas Satisfaccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D58D4D-5DE2-45DE-8A53-A1EF3865D9C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC396A9-296C-4707-AE06-B9C29F3C9B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B9009996-7F59-40D8-9537-CE1DA053594C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{B9009996-7F59-40D8-9537-CE1DA053594C}"/>
   </bookViews>
   <sheets>
     <sheet name="Objetos" sheetId="1" r:id="rId1"/>
-    <sheet name="Orden Paquetes" sheetId="2" r:id="rId2"/>
-    <sheet name="listas" sheetId="3" r:id="rId3"/>
+    <sheet name="Hoja2" sheetId="5" r:id="rId2"/>
+    <sheet name="Orden Paquetes" sheetId="2" r:id="rId3"/>
+    <sheet name="listas" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="TIPO_OBJETO">listas!$A$2:$A$8</definedName>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="59">
   <si>
     <t>NOMBRE TECNICO</t>
   </si>
@@ -215,13 +216,19 @@
   </si>
   <si>
     <t>04_MA_AWS_ENCUSATIS_01</t>
+  </si>
+  <si>
+    <t>03_SV_AWS_ENCUSATIS_02</t>
+  </si>
+  <si>
+    <t>Academica Encuestas Satisfacción 2.0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -239,6 +246,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -315,19 +329,24 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1184,7 +1203,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="33" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E33" s="4" t="str">
         <f>IFERROR(VLOOKUP(D33,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1194,7 +1213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="34" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E34" s="4" t="str">
         <f>IFERROR(VLOOKUP(D34,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1204,7 +1223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="35" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E35" s="4" t="str">
         <f>IFERROR(VLOOKUP(D35,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1214,7 +1233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="36" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E36" s="4" t="str">
         <f>IFERROR(VLOOKUP(D36,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1224,7 +1243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="37" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E37" s="4" t="str">
         <f>IFERROR(VLOOKUP(D37,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1234,7 +1253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="38" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E38" s="4" t="str">
         <f>IFERROR(VLOOKUP(D38,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1244,17 +1263,23 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="39" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>58</v>
+      </c>
+      <c r="C39" t="s">
+        <v>57</v>
+      </c>
       <c r="E39" s="4" t="str">
         <f>IFERROR(VLOOKUP(D39,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
       <c r="F39" s="5" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="40" spans="5:6" x14ac:dyDescent="0.25">
+        <v xml:space="preserve"> 03_SV_AWS_ENCUSATIS_02</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E40" s="4" t="str">
         <f>IFERROR(VLOOKUP(D40,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1264,7 +1289,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="41" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E41" s="4" t="str">
         <f>IFERROR(VLOOKUP(D41,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1274,7 +1299,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="42" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E42" s="4" t="str">
         <f>IFERROR(VLOOKUP(D42,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1284,7 +1309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="43" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E43" s="4" t="str">
         <f>IFERROR(VLOOKUP(D43,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1294,7 +1319,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="44" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E44" s="4" t="str">
         <f>IFERROR(VLOOKUP(D44,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1304,7 +1329,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="45" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E45" s="4" t="str">
         <f>IFERROR(VLOOKUP(D45,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1314,7 +1339,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="46" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E46" s="4" t="str">
         <f>IFERROR(VLOOKUP(D46,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1324,7 +1349,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="47" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E47" s="4" t="str">
         <f>IFERROR(VLOOKUP(D47,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1334,7 +1359,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="48" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
       <c r="E48" s="4" t="str">
         <f>IFERROR(VLOOKUP(D48,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1646,6 +1671,232 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9646EA99-A061-4937-BA82-2B3637E717DF}">
+  <dimension ref="A1:U5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>6863</v>
+      </c>
+      <c r="B1">
+        <v>8268</v>
+      </c>
+      <c r="C1">
+        <v>8463</v>
+      </c>
+      <c r="D1">
+        <v>12642</v>
+      </c>
+      <c r="E1">
+        <v>6651</v>
+      </c>
+      <c r="F1">
+        <v>5115</v>
+      </c>
+      <c r="H1">
+        <v>48002</v>
+      </c>
+      <c r="I1">
+        <v>11646</v>
+      </c>
+      <c r="J1">
+        <v>11825</v>
+      </c>
+      <c r="K1">
+        <v>46898</v>
+      </c>
+      <c r="L1">
+        <v>33959</v>
+      </c>
+      <c r="N1">
+        <v>11156</v>
+      </c>
+      <c r="O1">
+        <v>11156</v>
+      </c>
+      <c r="P1">
+        <v>1154</v>
+      </c>
+      <c r="Q1">
+        <v>135</v>
+      </c>
+      <c r="R1">
+        <v>4963</v>
+      </c>
+      <c r="S1">
+        <v>862</v>
+      </c>
+      <c r="T1" s="8"/>
+      <c r="U1">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1704</v>
+      </c>
+      <c r="B2">
+        <v>1955</v>
+      </c>
+      <c r="C2">
+        <v>1924</v>
+      </c>
+      <c r="D2">
+        <v>2907</v>
+      </c>
+      <c r="E2">
+        <v>1512</v>
+      </c>
+      <c r="F2">
+        <v>1154</v>
+      </c>
+      <c r="H2">
+        <v>11156</v>
+      </c>
+      <c r="I2">
+        <v>2666</v>
+      </c>
+      <c r="J2">
+        <v>2666</v>
+      </c>
+      <c r="K2">
+        <v>11156</v>
+      </c>
+      <c r="L2">
+        <v>7497</v>
+      </c>
+      <c r="N2">
+        <v>135</v>
+      </c>
+      <c r="O2">
+        <v>397</v>
+      </c>
+      <c r="P2">
+        <v>16</v>
+      </c>
+      <c r="Q2">
+        <v>397</v>
+      </c>
+      <c r="R2">
+        <v>5119</v>
+      </c>
+      <c r="S2">
+        <v>1541</v>
+      </c>
+      <c r="T2" s="8"/>
+      <c r="U2">
+        <v>2666</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
+        <f>+A1/A2</f>
+        <v>4.027582159624413</v>
+      </c>
+      <c r="B3" s="6">
+        <f>+B1/B2</f>
+        <v>4.2291560102301791</v>
+      </c>
+      <c r="C3" s="6">
+        <f t="shared" ref="C3:F3" si="0">+C1/C2</f>
+        <v>4.3986486486486482</v>
+      </c>
+      <c r="D3" s="6">
+        <f t="shared" si="0"/>
+        <v>4.3488132094943239</v>
+      </c>
+      <c r="E3" s="6">
+        <f t="shared" si="0"/>
+        <v>4.3988095238095237</v>
+      </c>
+      <c r="F3" s="6">
+        <f t="shared" si="0"/>
+        <v>4.4324090121317159</v>
+      </c>
+      <c r="H3" s="6">
+        <f>+H1/H2</f>
+        <v>4.3027967013266402</v>
+      </c>
+      <c r="I3" s="6">
+        <f>+I1/I2</f>
+        <v>4.3683420855213804</v>
+      </c>
+      <c r="J3" s="6">
+        <f>+J1/J2</f>
+        <v>4.435483870967742</v>
+      </c>
+      <c r="K3" s="6">
+        <f>+K1/K2</f>
+        <v>4.2038365005378271</v>
+      </c>
+      <c r="L3" s="6">
+        <f>+L1/L2</f>
+        <v>4.5296785380818996</v>
+      </c>
+      <c r="N3" s="7">
+        <f>+N2/N1</f>
+        <v>1.2101111509501614E-2</v>
+      </c>
+      <c r="O3" s="7">
+        <f>+O2/O1</f>
+        <v>3.5586231624238081E-2</v>
+      </c>
+      <c r="P3" s="7">
+        <f>+P2/P1</f>
+        <v>1.3864818024263431E-2</v>
+      </c>
+      <c r="Q3">
+        <f>+Q2+Q1</f>
+        <v>532</v>
+      </c>
+      <c r="R3">
+        <f>+R2+R1</f>
+        <v>10082</v>
+      </c>
+      <c r="S3">
+        <f>+S2+S1</f>
+        <v>2403</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="Q4">
+        <v>11156</v>
+      </c>
+      <c r="R4">
+        <v>11156</v>
+      </c>
+      <c r="S4">
+        <v>2666</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="Q5" s="7">
+        <f>+Q3/Q4</f>
+        <v>4.7687343133739693E-2</v>
+      </c>
+      <c r="R5" s="7">
+        <f>+R3/R4</f>
+        <v>0.90372893510218721</v>
+      </c>
+      <c r="S5" s="7">
+        <f>+S3/S4</f>
+        <v>0.90135033758439609</v>
+      </c>
+      <c r="U5" s="7">
+        <f>+U1/U2</f>
+        <v>1.2378094523630907E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C75E2AA2-5432-4E9C-93A9-C36766097F89}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1718,7 +1969,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6E318EA-3F07-4D83-8AAC-62F6B6937B60}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
se carga archivos 28_04_2026
</commit_message>
<xml_diff>
--- a/DataSphere/Encuestas Satisfaccion/Formato Objetos Transporte Ajustes Encuestas Satisfacción.xlsx
+++ b/DataSphere/Encuestas Satisfaccion/Formato Objetos Transporte Ajustes Encuestas Satisfacción.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\degonzalez\Documents\2026\Backup_2026\DataSphere\Encuestas Satisfaccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC396A9-296C-4707-AE06-B9C29F3C9B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4BC2FA-9D59-4E3E-8592-C37EAF1026A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{B9009996-7F59-40D8-9537-CE1DA053594C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B9009996-7F59-40D8-9537-CE1DA053594C}"/>
   </bookViews>
   <sheets>
     <sheet name="Objetos" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="60">
   <si>
     <t>NOMBRE TECNICO</t>
   </si>
@@ -206,12 +206,6 @@
     <t>02_DF_AWS_ENCUSATIS2024_02</t>
   </si>
   <si>
-    <t>Academica Encuestas Satisfacción</t>
-  </si>
-  <si>
-    <t>03_SV_AWS_ENCUSATIS_01</t>
-  </si>
-  <si>
     <t>Bussines Inteligence/Tableros/Experiencia Estudiantil/Encuestas Satisfaccion/</t>
   </si>
   <si>
@@ -221,7 +215,16 @@
     <t>03_SV_AWS_ENCUSATIS_02</t>
   </si>
   <si>
-    <t>Academica Encuestas Satisfacción 2.0</t>
+    <t>Academia Encuestas Satisfacción 2.0</t>
+  </si>
+  <si>
+    <t>Academia Encuestas Satisfacción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mediaciones Encuestas Satisfacción </t>
+  </si>
+  <si>
+    <t>03_SV_AWS_MEDIACIONES_01</t>
   </si>
 </sst>
 </file>
@@ -682,7 +685,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="2" max="2" width="38.140625" customWidth="1"/>
     <col min="3" max="3" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.140625" customWidth="1"/>
     <col min="5" max="5" width="21.140625" style="4" customWidth="1"/>
@@ -1011,10 +1014,10 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D16" t="s">
         <v>30</v>
@@ -1025,18 +1028,18 @@
       </c>
       <c r="F16" s="5" t="str">
         <f t="shared" si="1"/>
-        <v>SV 03_SV_AWS_ENCUSATIS_01</v>
+        <v>SV 03_SV_AWS_ENCUSATIS_02</v>
       </c>
       <c r="G16" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C17" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D17" t="s">
         <v>6</v>
@@ -1050,17 +1053,29 @@
         <v>AM 04_MA_AWS_ENCUSATIS_01</v>
       </c>
       <c r="G17" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
       <c r="E18" s="4" t="str">
         <f>IFERROR(VLOOKUP(D18,listas!$A$2:$B$8,2,0),"")</f>
-        <v/>
+        <v>SV</v>
       </c>
       <c r="F18" s="5" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+        <v>SV 03_SV_AWS_MEDIACIONES_01</v>
+      </c>
+      <c r="G18" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
@@ -1203,7 +1218,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E33" s="4" t="str">
         <f>IFERROR(VLOOKUP(D33,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1213,7 +1228,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E34" s="4" t="str">
         <f>IFERROR(VLOOKUP(D34,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1223,7 +1238,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E35" s="4" t="str">
         <f>IFERROR(VLOOKUP(D35,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1233,7 +1248,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E36" s="4" t="str">
         <f>IFERROR(VLOOKUP(D36,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1243,7 +1258,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E37" s="4" t="str">
         <f>IFERROR(VLOOKUP(D37,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1253,7 +1268,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E38" s="4" t="str">
         <f>IFERROR(VLOOKUP(D38,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1263,23 +1278,17 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B39" t="s">
-        <v>58</v>
-      </c>
-      <c r="C39" t="s">
-        <v>57</v>
-      </c>
+    <row r="39" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E39" s="4" t="str">
         <f>IFERROR(VLOOKUP(D39,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
       <c r="F39" s="5" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> 03_SV_AWS_ENCUSATIS_02</v>
-      </c>
-    </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="40" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E40" s="4" t="str">
         <f>IFERROR(VLOOKUP(D40,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1289,7 +1298,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E41" s="4" t="str">
         <f>IFERROR(VLOOKUP(D41,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1299,7 +1308,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E42" s="4" t="str">
         <f>IFERROR(VLOOKUP(D42,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1309,7 +1318,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E43" s="4" t="str">
         <f>IFERROR(VLOOKUP(D43,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1319,7 +1328,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E44" s="4" t="str">
         <f>IFERROR(VLOOKUP(D44,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1329,7 +1338,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E45" s="4" t="str">
         <f>IFERROR(VLOOKUP(D45,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1339,7 +1348,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E46" s="4" t="str">
         <f>IFERROR(VLOOKUP(D46,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1349,7 +1358,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E47" s="4" t="str">
         <f>IFERROR(VLOOKUP(D47,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1359,7 +1368,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E48" s="4" t="str">
         <f>IFERROR(VLOOKUP(D48,listas!$A$2:$B$8,2,0),"")</f>
         <v/>

</xml_diff>

<commit_message>
se carga archivos nombres encuestas
</commit_message>
<xml_diff>
--- a/DataSphere/Encuestas Satisfaccion/Formato Objetos Transporte Ajustes Encuestas Satisfacción.xlsx
+++ b/DataSphere/Encuestas Satisfaccion/Formato Objetos Transporte Ajustes Encuestas Satisfacción.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\degonzalez\Documents\2026\Backup_2026\DataSphere\Encuestas Satisfaccion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Favorites\Daniel\Backup_2026\DataSphere\Encuestas Satisfaccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4BC2FA-9D59-4E3E-8592-C37EAF1026A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5299F93D-20AC-4AEC-BBC3-5A0E6E3BB99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B9009996-7F59-40D8-9537-CE1DA053594C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B9009996-7F59-40D8-9537-CE1DA053594C}"/>
   </bookViews>
   <sheets>
     <sheet name="Objetos" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="65">
   <si>
     <t>NOMBRE TECNICO</t>
   </si>
@@ -225,6 +225,21 @@
   </si>
   <si>
     <t>03_SV_AWS_MEDIACIONES_01</t>
+  </si>
+  <si>
+    <t>04_MA_AWS_MEDIACIONES_01</t>
+  </si>
+  <si>
+    <t>Mediaciones Encuestas Satisfacción</t>
+  </si>
+  <si>
+    <t>03_SV_AWS_FATLAB_01</t>
+  </si>
+  <si>
+    <t>Fatlab,Impacta y Sostenibilidad</t>
+  </si>
+  <si>
+    <t>04_MA_AWS_FATLAB_01</t>
   </si>
 </sst>
 </file>
@@ -336,7 +351,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -346,6 +361,9 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -682,18 +700,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED66D76B-AB7C-48E0-8218-0FCDF9992D65}">
   <dimension ref="A1:G79"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" customWidth="1"/>
-    <col min="2" max="2" width="38.140625" customWidth="1"/>
-    <col min="3" max="3" width="32.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.140625" customWidth="1"/>
-    <col min="5" max="5" width="21.140625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="21.453125" customWidth="1"/>
+    <col min="2" max="2" width="38.1796875" customWidth="1"/>
+    <col min="3" max="3" width="32.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.1796875" customWidth="1"/>
+    <col min="5" max="5" width="21.1796875" style="4" customWidth="1"/>
     <col min="6" max="6" width="34" style="5" customWidth="1"/>
-    <col min="7" max="7" width="69.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="69.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -716,7 +734,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>49</v>
       </c>
@@ -738,7 +756,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>38</v>
       </c>
@@ -760,7 +778,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>38</v>
       </c>
@@ -782,7 +800,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>33</v>
       </c>
@@ -804,7 +822,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>33</v>
       </c>
@@ -826,7 +844,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>34</v>
       </c>
@@ -848,7 +866,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>34</v>
       </c>
@@ -870,7 +888,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>35</v>
       </c>
@@ -892,7 +910,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>35</v>
       </c>
@@ -914,7 +932,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>36</v>
       </c>
@@ -936,7 +954,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>36</v>
       </c>
@@ -958,7 +976,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>37</v>
       </c>
@@ -980,7 +998,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>37</v>
       </c>
@@ -1002,7 +1020,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="E15" s="4" t="str">
         <f>IFERROR(VLOOKUP(D15,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1012,7 +1030,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>56</v>
       </c>
@@ -1034,7 +1052,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>57</v>
       </c>
@@ -1056,7 +1074,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>58</v>
       </c>
@@ -1078,37 +1096,64 @@
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B19" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" t="s">
+        <v>6</v>
+      </c>
       <c r="E19" s="4" t="str">
         <f>IFERROR(VLOOKUP(D19,listas!$A$2:$B$8,2,0),"")</f>
-        <v/>
+        <v>AM</v>
       </c>
       <c r="F19" s="5" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+        <v>AM 04_MA_AWS_MEDIACIONES_01</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" t="s">
+        <v>62</v>
+      </c>
+      <c r="D20" t="s">
+        <v>30</v>
+      </c>
       <c r="E20" s="4" t="str">
         <f>IFERROR(VLOOKUP(D20,listas!$A$2:$B$8,2,0),"")</f>
-        <v/>
+        <v>SV</v>
       </c>
       <c r="F20" s="5" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+        <v>SV 03_SV_AWS_FATLAB_01</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
+        <v>63</v>
+      </c>
+      <c r="C21" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" t="s">
+        <v>6</v>
+      </c>
       <c r="E21" s="4" t="str">
         <f>IFERROR(VLOOKUP(D21,listas!$A$2:$B$8,2,0),"")</f>
-        <v/>
+        <v>AM</v>
       </c>
       <c r="F21" s="5" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+        <v>AM 04_MA_AWS_FATLAB_01</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E22" s="4" t="str">
         <f>IFERROR(VLOOKUP(D22,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1118,7 +1163,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E23" s="4" t="str">
         <f>IFERROR(VLOOKUP(D23,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1128,7 +1173,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E24" s="4" t="str">
         <f>IFERROR(VLOOKUP(D24,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1138,7 +1183,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E25" s="4" t="str">
         <f>IFERROR(VLOOKUP(D25,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1148,7 +1193,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E26" s="4" t="str">
         <f>IFERROR(VLOOKUP(D26,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1158,7 +1203,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E27" s="4" t="str">
         <f>IFERROR(VLOOKUP(D27,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1168,7 +1213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E28" s="4" t="str">
         <f>IFERROR(VLOOKUP(D28,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1178,7 +1223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E29" s="4" t="str">
         <f>IFERROR(VLOOKUP(D29,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1188,7 +1233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E30" s="4" t="str">
         <f>IFERROR(VLOOKUP(D30,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1198,7 +1243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E31" s="4" t="str">
         <f>IFERROR(VLOOKUP(D31,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1208,7 +1253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
       <c r="E32" s="4" t="str">
         <f>IFERROR(VLOOKUP(D32,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1218,7 +1263,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="33" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E33" s="4" t="str">
         <f>IFERROR(VLOOKUP(D33,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1228,7 +1273,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="34" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E34" s="4" t="str">
         <f>IFERROR(VLOOKUP(D34,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1238,7 +1283,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="35" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E35" s="4" t="str">
         <f>IFERROR(VLOOKUP(D35,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1248,7 +1293,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="36" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E36" s="4" t="str">
         <f>IFERROR(VLOOKUP(D36,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1258,7 +1303,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="37" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E37" s="4" t="str">
         <f>IFERROR(VLOOKUP(D37,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1268,7 +1313,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="38" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E38" s="4" t="str">
         <f>IFERROR(VLOOKUP(D38,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1278,7 +1323,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="39" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E39" s="4" t="str">
         <f>IFERROR(VLOOKUP(D39,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1288,7 +1333,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="40" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E40" s="4" t="str">
         <f>IFERROR(VLOOKUP(D40,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1298,7 +1343,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="41" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E41" s="4" t="str">
         <f>IFERROR(VLOOKUP(D41,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1308,7 +1353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="42" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E42" s="4" t="str">
         <f>IFERROR(VLOOKUP(D42,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1318,7 +1363,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="43" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E43" s="4" t="str">
         <f>IFERROR(VLOOKUP(D43,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1328,7 +1373,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="44" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E44" s="4" t="str">
         <f>IFERROR(VLOOKUP(D44,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1338,7 +1383,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="45" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E45" s="4" t="str">
         <f>IFERROR(VLOOKUP(D45,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1348,7 +1393,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="46" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E46" s="4" t="str">
         <f>IFERROR(VLOOKUP(D46,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1358,7 +1403,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="47" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E47" s="4" t="str">
         <f>IFERROR(VLOOKUP(D47,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1368,7 +1413,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="48" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E48" s="4" t="str">
         <f>IFERROR(VLOOKUP(D48,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1378,7 +1423,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="49" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E49" s="4" t="str">
         <f>IFERROR(VLOOKUP(D49,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1388,7 +1433,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="50" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E50" s="4" t="str">
         <f>IFERROR(VLOOKUP(D50,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1398,7 +1443,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="51" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E51" s="4" t="str">
         <f>IFERROR(VLOOKUP(D51,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1408,7 +1453,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="52" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E52" s="4" t="str">
         <f>IFERROR(VLOOKUP(D52,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1418,7 +1463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="53" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E53" s="4" t="str">
         <f>IFERROR(VLOOKUP(D53,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1428,7 +1473,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="54" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E54" s="4" t="str">
         <f>IFERROR(VLOOKUP(D54,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1438,7 +1483,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="55" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E55" s="4" t="str">
         <f>IFERROR(VLOOKUP(D55,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1448,7 +1493,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="56" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E56" s="4" t="str">
         <f>IFERROR(VLOOKUP(D56,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1458,7 +1503,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="57" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E57" s="4" t="str">
         <f>IFERROR(VLOOKUP(D57,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1468,7 +1513,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="58" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E58" s="4" t="str">
         <f>IFERROR(VLOOKUP(D58,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1478,7 +1523,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="59" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E59" s="4" t="str">
         <f>IFERROR(VLOOKUP(D59,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1488,7 +1533,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="60" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E60" s="4" t="str">
         <f>IFERROR(VLOOKUP(D60,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1498,7 +1543,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="61" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E61" s="4" t="str">
         <f>IFERROR(VLOOKUP(D61,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1508,7 +1553,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="62" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E62" s="4" t="str">
         <f>IFERROR(VLOOKUP(D62,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1518,7 +1563,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="63" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E63" s="4" t="str">
         <f>IFERROR(VLOOKUP(D63,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1528,7 +1573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="64" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E64" s="4" t="str">
         <f>IFERROR(VLOOKUP(D64,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1538,7 +1583,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="65" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E65" s="4" t="str">
         <f>IFERROR(VLOOKUP(D65,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1548,7 +1593,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="66" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E66" s="4" t="str">
         <f>IFERROR(VLOOKUP(D66,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1558,7 +1603,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="67" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E67" s="4" t="str">
         <f>IFERROR(VLOOKUP(D67,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1568,7 +1613,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="68" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E68" s="4" t="str">
         <f>IFERROR(VLOOKUP(D68,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1578,7 +1623,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="69" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E69" s="4" t="str">
         <f>IFERROR(VLOOKUP(D69,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1588,7 +1633,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="70" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E70" s="4" t="str">
         <f>IFERROR(VLOOKUP(D70,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1598,7 +1643,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="71" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E71" s="4" t="str">
         <f>IFERROR(VLOOKUP(D71,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1608,7 +1653,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="72" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E72" s="4" t="str">
         <f>IFERROR(VLOOKUP(D72,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1618,7 +1663,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="73" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E73" s="4" t="str">
         <f>IFERROR(VLOOKUP(D73,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1628,7 +1673,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="74" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E74" s="4" t="str">
         <f>IFERROR(VLOOKUP(D74,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1638,31 +1683,31 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="75" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E75" s="4" t="str">
         <f>IFERROR(VLOOKUP(D75,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
     </row>
-    <row r="76" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E76" s="4" t="str">
         <f>IFERROR(VLOOKUP(D76,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
     </row>
-    <row r="77" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E77" s="4" t="str">
         <f>IFERROR(VLOOKUP(D77,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
     </row>
-    <row r="78" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E78" s="4" t="str">
         <f>IFERROR(VLOOKUP(D78,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
     </row>
-    <row r="79" spans="5:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="5:6" x14ac:dyDescent="0.35">
       <c r="E79" s="4" t="str">
         <f>IFERROR(VLOOKUP(D79,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1682,12 +1727,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9646EA99-A061-4937-BA82-2B3637E717DF}">
   <dimension ref="A1:U5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1">
         <v>6863</v>
       </c>
@@ -1744,7 +1789,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1704</v>
       </c>
@@ -1801,7 +1846,7 @@
         <v>2666</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" s="6">
         <f>+A1/A2</f>
         <v>4.027582159624413</v>
@@ -1871,7 +1916,7 @@
         <v>2403</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="Q4">
         <v>11156</v>
       </c>
@@ -1882,7 +1927,7 @@
         <v>2666</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="Q5" s="7">
         <f>+Q3/Q4</f>
         <v>4.7687343133739693E-2</v>
@@ -1908,17 +1953,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C75E2AA2-5432-4E9C-93A9-C36766097F89}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="41.42578125" customWidth="1"/>
+    <col min="2" max="2" width="41.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1929,7 +1974,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -1940,7 +1985,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -1951,7 +1996,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -1962,7 +2007,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -1981,13 +2026,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6E318EA-3F07-4D83-8AAC-62F6B6937B60}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="36.140625" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" customWidth="1"/>
+    <col min="1" max="1" width="36.1796875" customWidth="1"/>
+    <col min="2" max="2" width="23.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -1995,7 +2040,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -2003,7 +2048,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2011,7 +2056,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -2019,7 +2064,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -2027,7 +2072,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -2035,7 +2080,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -2043,7 +2088,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>30</v>
       </c>

</xml_diff>

<commit_message>
se cargan archivos 08_05_2026
</commit_message>
<xml_diff>
--- a/DataSphere/Encuestas Satisfaccion/Formato Objetos Transporte Ajustes Encuestas Satisfacción.xlsx
+++ b/DataSphere/Encuestas Satisfaccion/Formato Objetos Transporte Ajustes Encuestas Satisfacción.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Favorites\Daniel\Backup_2026\DataSphere\Encuestas Satisfaccion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\degonzalez\Documents\2026\Backup_2026\DataSphere\Encuestas Satisfaccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5299F93D-20AC-4AEC-BBC3-5A0E6E3BB99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D4B8242-CB2A-4797-A474-2F5D7A4CBAAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B9009996-7F59-40D8-9537-CE1DA053594C}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B9009996-7F59-40D8-9537-CE1DA053594C}"/>
   </bookViews>
   <sheets>
     <sheet name="Objetos" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="68">
   <si>
     <t>NOMBRE TECNICO</t>
   </si>
@@ -240,6 +240,15 @@
   </si>
   <si>
     <t>04_MA_AWS_FATLAB_01</t>
+  </si>
+  <si>
+    <t>04_MA_AWS_NPS_SATIS_01</t>
+  </si>
+  <si>
+    <t>Nps Satisfacción Estudiantes</t>
+  </si>
+  <si>
+    <t>03_SV_AWS_NPS_SATIS_01</t>
   </si>
 </sst>
 </file>
@@ -700,18 +709,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED66D76B-AB7C-48E0-8218-0FCDF9992D65}">
   <dimension ref="A1:G79"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.453125" customWidth="1"/>
-    <col min="2" max="2" width="38.1796875" customWidth="1"/>
-    <col min="3" max="3" width="32.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.1796875" customWidth="1"/>
-    <col min="5" max="5" width="21.1796875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="2" max="2" width="38.140625" customWidth="1"/>
+    <col min="3" max="3" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" customWidth="1"/>
+    <col min="5" max="5" width="21.140625" style="4" customWidth="1"/>
     <col min="6" max="6" width="34" style="5" customWidth="1"/>
-    <col min="7" max="7" width="69.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="69.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -734,7 +743,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>49</v>
       </c>
@@ -756,7 +765,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>38</v>
       </c>
@@ -778,7 +787,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>38</v>
       </c>
@@ -800,7 +809,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>33</v>
       </c>
@@ -822,7 +831,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>33</v>
       </c>
@@ -844,7 +853,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>34</v>
       </c>
@@ -866,7 +875,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>34</v>
       </c>
@@ -888,7 +897,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>35</v>
       </c>
@@ -910,7 +919,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>35</v>
       </c>
@@ -932,7 +941,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>36</v>
       </c>
@@ -954,7 +963,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>36</v>
       </c>
@@ -976,7 +985,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>37</v>
       </c>
@@ -998,7 +1007,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>37</v>
       </c>
@@ -1020,7 +1029,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E15" s="4" t="str">
         <f>IFERROR(VLOOKUP(D15,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1030,7 +1039,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>56</v>
       </c>
@@ -1052,7 +1061,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>57</v>
       </c>
@@ -1074,7 +1083,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>58</v>
       </c>
@@ -1096,7 +1105,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="9" t="s">
         <v>61</v>
       </c>
@@ -1114,8 +1123,11 @@
         <f t="shared" si="1"/>
         <v>AM 04_MA_AWS_MEDIACIONES_01</v>
       </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="G19" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>63</v>
       </c>
@@ -1133,8 +1145,11 @@
         <f t="shared" si="1"/>
         <v>SV 03_SV_AWS_FATLAB_01</v>
       </c>
-    </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="G20" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>63</v>
       </c>
@@ -1152,28 +1167,55 @@
         <f t="shared" si="1"/>
         <v>AM 04_MA_AWS_FATLAB_01</v>
       </c>
-    </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="G21" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" t="s">
+        <v>67</v>
+      </c>
+      <c r="D22" t="s">
+        <v>30</v>
+      </c>
       <c r="E22" s="4" t="str">
         <f>IFERROR(VLOOKUP(D22,listas!$A$2:$B$8,2,0),"")</f>
-        <v/>
+        <v>SV</v>
       </c>
       <c r="F22" s="5" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.35">
+        <v>SV 03_SV_AWS_NPS_SATIS_01</v>
+      </c>
+      <c r="G22" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" t="s">
+        <v>6</v>
+      </c>
       <c r="E23" s="4" t="str">
         <f>IFERROR(VLOOKUP(D23,listas!$A$2:$B$8,2,0),"")</f>
-        <v/>
+        <v>AM</v>
       </c>
       <c r="F23" s="5" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
+        <v>AM 04_MA_AWS_NPS_SATIS_01</v>
+      </c>
+      <c r="G23" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E24" s="4" t="str">
         <f>IFERROR(VLOOKUP(D24,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1183,7 +1225,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E25" s="4" t="str">
         <f>IFERROR(VLOOKUP(D25,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1193,7 +1235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E26" s="4" t="str">
         <f>IFERROR(VLOOKUP(D26,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1203,7 +1245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E27" s="4" t="str">
         <f>IFERROR(VLOOKUP(D27,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1213,7 +1255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E28" s="4" t="str">
         <f>IFERROR(VLOOKUP(D28,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1223,7 +1265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E29" s="4" t="str">
         <f>IFERROR(VLOOKUP(D29,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1233,7 +1275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E30" s="4" t="str">
         <f>IFERROR(VLOOKUP(D30,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1243,7 +1285,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E31" s="4" t="str">
         <f>IFERROR(VLOOKUP(D31,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1253,7 +1295,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="E32" s="4" t="str">
         <f>IFERROR(VLOOKUP(D32,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1263,7 +1305,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="33" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E33" s="4" t="str">
         <f>IFERROR(VLOOKUP(D33,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1273,7 +1315,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="34" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E34" s="4" t="str">
         <f>IFERROR(VLOOKUP(D34,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1283,7 +1325,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="35" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E35" s="4" t="str">
         <f>IFERROR(VLOOKUP(D35,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1293,7 +1335,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="36" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E36" s="4" t="str">
         <f>IFERROR(VLOOKUP(D36,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1303,7 +1345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="37" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E37" s="4" t="str">
         <f>IFERROR(VLOOKUP(D37,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1313,7 +1355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="38" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E38" s="4" t="str">
         <f>IFERROR(VLOOKUP(D38,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1323,7 +1365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="39" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E39" s="4" t="str">
         <f>IFERROR(VLOOKUP(D39,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1333,7 +1375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="40" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E40" s="4" t="str">
         <f>IFERROR(VLOOKUP(D40,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1343,7 +1385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="41" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E41" s="4" t="str">
         <f>IFERROR(VLOOKUP(D41,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1353,7 +1395,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="42" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E42" s="4" t="str">
         <f>IFERROR(VLOOKUP(D42,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1363,7 +1405,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="43" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E43" s="4" t="str">
         <f>IFERROR(VLOOKUP(D43,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1373,7 +1415,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="44" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E44" s="4" t="str">
         <f>IFERROR(VLOOKUP(D44,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1383,7 +1425,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="45" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E45" s="4" t="str">
         <f>IFERROR(VLOOKUP(D45,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1393,7 +1435,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="46" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E46" s="4" t="str">
         <f>IFERROR(VLOOKUP(D46,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1403,7 +1445,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="47" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E47" s="4" t="str">
         <f>IFERROR(VLOOKUP(D47,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1413,7 +1455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="48" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E48" s="4" t="str">
         <f>IFERROR(VLOOKUP(D48,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1423,7 +1465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="49" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E49" s="4" t="str">
         <f>IFERROR(VLOOKUP(D49,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1433,7 +1475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="50" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E50" s="4" t="str">
         <f>IFERROR(VLOOKUP(D50,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1443,7 +1485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="51" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E51" s="4" t="str">
         <f>IFERROR(VLOOKUP(D51,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1453,7 +1495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="52" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E52" s="4" t="str">
         <f>IFERROR(VLOOKUP(D52,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1463,7 +1505,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="53" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E53" s="4" t="str">
         <f>IFERROR(VLOOKUP(D53,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1473,7 +1515,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="54" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E54" s="4" t="str">
         <f>IFERROR(VLOOKUP(D54,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1483,7 +1525,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="55" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E55" s="4" t="str">
         <f>IFERROR(VLOOKUP(D55,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1493,7 +1535,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="56" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E56" s="4" t="str">
         <f>IFERROR(VLOOKUP(D56,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1503,7 +1545,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="57" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E57" s="4" t="str">
         <f>IFERROR(VLOOKUP(D57,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1513,7 +1555,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="58" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E58" s="4" t="str">
         <f>IFERROR(VLOOKUP(D58,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1523,7 +1565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="59" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E59" s="4" t="str">
         <f>IFERROR(VLOOKUP(D59,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1533,7 +1575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="60" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E60" s="4" t="str">
         <f>IFERROR(VLOOKUP(D60,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1543,7 +1585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="61" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E61" s="4" t="str">
         <f>IFERROR(VLOOKUP(D61,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1553,7 +1595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="62" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E62" s="4" t="str">
         <f>IFERROR(VLOOKUP(D62,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1563,7 +1605,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="63" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E63" s="4" t="str">
         <f>IFERROR(VLOOKUP(D63,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1573,7 +1615,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="64" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E64" s="4" t="str">
         <f>IFERROR(VLOOKUP(D64,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1583,7 +1625,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="65" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E65" s="4" t="str">
         <f>IFERROR(VLOOKUP(D65,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1593,7 +1635,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="66" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E66" s="4" t="str">
         <f>IFERROR(VLOOKUP(D66,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1603,7 +1645,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="67" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E67" s="4" t="str">
         <f>IFERROR(VLOOKUP(D67,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1613,7 +1655,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="68" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="68" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E68" s="4" t="str">
         <f>IFERROR(VLOOKUP(D68,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1623,7 +1665,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="69" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="69" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E69" s="4" t="str">
         <f>IFERROR(VLOOKUP(D69,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1633,7 +1675,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="70" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="70" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E70" s="4" t="str">
         <f>IFERROR(VLOOKUP(D70,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1643,7 +1685,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="71" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="71" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E71" s="4" t="str">
         <f>IFERROR(VLOOKUP(D71,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1653,7 +1695,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="72" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="72" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E72" s="4" t="str">
         <f>IFERROR(VLOOKUP(D72,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1663,7 +1705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="73" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="73" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E73" s="4" t="str">
         <f>IFERROR(VLOOKUP(D73,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1673,7 +1715,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="74" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="74" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E74" s="4" t="str">
         <f>IFERROR(VLOOKUP(D74,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1683,31 +1725,31 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="75" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="75" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E75" s="4" t="str">
         <f>IFERROR(VLOOKUP(D75,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
     </row>
-    <row r="76" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E76" s="4" t="str">
         <f>IFERROR(VLOOKUP(D76,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
     </row>
-    <row r="77" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E77" s="4" t="str">
         <f>IFERROR(VLOOKUP(D77,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
     </row>
-    <row r="78" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E78" s="4" t="str">
         <f>IFERROR(VLOOKUP(D78,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
       </c>
     </row>
-    <row r="79" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E79" s="4" t="str">
         <f>IFERROR(VLOOKUP(D79,listas!$A$2:$B$8,2,0),"")</f>
         <v/>
@@ -1715,7 +1757,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D44" xr:uid="{4E78058F-6DE9-4785-B4B6-576D9F0A6DEF}">
       <formula1>TIPO_OBJETO</formula1>
     </dataValidation>
@@ -1727,12 +1769,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9646EA99-A061-4937-BA82-2B3637E717DF}">
   <dimension ref="A1:U5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1">
         <v>6863</v>
       </c>
@@ -1789,7 +1831,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1704</v>
       </c>
@@ -1846,7 +1888,7 @@
         <v>2666</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="6">
         <f>+A1/A2</f>
         <v>4.027582159624413</v>
@@ -1916,7 +1958,7 @@
         <v>2403</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="Q4">
         <v>11156</v>
       </c>
@@ -1927,7 +1969,7 @@
         <v>2666</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="Q5" s="7">
         <f>+Q3/Q4</f>
         <v>4.7687343133739693E-2</v>
@@ -1953,17 +1995,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C75E2AA2-5432-4E9C-93A9-C36766097F89}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="41.453125" customWidth="1"/>
+    <col min="2" max="2" width="41.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1974,7 +2016,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -1985,7 +2027,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -1996,7 +2038,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -2007,7 +2049,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -2026,13 +2068,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6E318EA-3F07-4D83-8AAC-62F6B6937B60}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.1796875" customWidth="1"/>
-    <col min="2" max="2" width="23.81640625" customWidth="1"/>
+    <col min="1" max="1" width="36.140625" customWidth="1"/>
+    <col min="2" max="2" width="23.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -2040,7 +2082,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -2048,7 +2090,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2056,7 +2098,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -2064,7 +2106,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -2072,7 +2114,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -2080,7 +2122,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -2088,7 +2130,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>30</v>
       </c>

</xml_diff>